<commit_message>
scan: seg6 2026-08-13 18:20 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-08-13.xlsx
+++ b/output/full_scan/batch_seq7_2026-08-13.xlsx
@@ -1799,21 +1799,21 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6739</v>
+        <v>6781</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>竹陞科技</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>565.3791324728163</v>
+        <v>531.6388249963093</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1045</v>
+        <v>1125</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>49.84933386412813</v>
+        <v>55.75784496279339</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>10.48224890951374</v>
+        <v>21.70772131656243</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.652710967577269</v>
+        <v>0.6812075675506158</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,48 +1842,48 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>13.69369593672724</v>
+        <v>27.29617318376082</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, kd_golden_cross, obv_uptrend, dealer_buy_3d</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6781</v>
+        <v>6806</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>森崴能源</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>531.6388249963093</v>
+        <v>528.7768356926886</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1125</v>
+        <v>3.51</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G27" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>55.75784496279339</v>
+        <v>31.69502796334339</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>21.70772131656243</v>
+        <v>32.59319934807885</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.6812075675506158</v>
+        <v>2.013053626871306</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,48 +1895,48 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>27.29617318376082</v>
+        <v>0.4112821325422744</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6806</v>
+        <v>6532</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>森崴能源</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>528.7768356926886</v>
+        <v>523.7756801768195</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>3.51</v>
+        <v>87</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G28" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>31.69502796334339</v>
+        <v>65.77557388116138</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>32.59319934807885</v>
+        <v>28.7461264035022</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>2.013053626871306</v>
+        <v>1.129839418574075</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.4112821325422744</v>
+        <v>3.03091793050582</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6532</v>
+        <v>6788</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>523.7756801768195</v>
+        <v>520.9223478213482</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>87</v>
+        <v>363.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>65.77557388116138</v>
+        <v>50.67999385264918</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.7461264035022</v>
+        <v>27.76190100228168</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.129839418574075</v>
+        <v>0.572899931983292</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.03091793050582</v>
+        <v>6.60832176381339</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6788</v>
+        <v>6597</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>520.9223478213482</v>
+        <v>513.6677251862392</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>363.5</v>
+        <v>68</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.67999385264918</v>
+        <v>52.29117596276318</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>27.76190100228168</v>
+        <v>9.514012647957021</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.572899931983292</v>
+        <v>0.8444742466786808</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>6.60832176381339</v>
+        <v>0.0669386584714044</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
+          <t>macd_golden_cross, breakout_20d, market_above_ma60, avoid_chase, hist_turn_positive, obv_uptrend, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6597</v>
+        <v>6805</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>513.6677251862392</v>
+        <v>505.0779235069686</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>68</v>
+        <v>1830</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>52.29117596276318</v>
+        <v>63.78878098099401</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>9.514012647957021</v>
+        <v>30.85367740059933</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.8444742466786808</v>
+        <v>1.27496456745889</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0669386584714044</v>
+        <v>58.5531809976468</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, breakout_20d, market_above_ma60, avoid_chase, hist_turn_positive, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6805</v>
+        <v>6807</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>505.0779235069686</v>
+        <v>502.5762420098295</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1830</v>
+        <v>38</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>63.78878098099401</v>
+        <v>74.45528723082759</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>30.85367740059933</v>
+        <v>20.68179010771956</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.27496456745889</v>
+        <v>1.029481049328883</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>58.5531809976468</v>
+        <v>0.3680262636577937</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6807</v>
+        <v>6584</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>502.5762420098295</v>
+        <v>498.8866495798871</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>38</v>
+        <v>597</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>74.45528723082759</v>
+        <v>57.26355097386514</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>20.68179010771956</v>
+        <v>25.97599744240152</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.029481049328883</v>
+        <v>0.9192835670113714</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3680262636577937</v>
+        <v>16.55457207208008</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6584</v>
+        <v>6727</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>亞泰金屬</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>498.8866495798871</v>
+        <v>498.5467088339622</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>597</v>
+        <v>393</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.26355097386514</v>
+        <v>51.03994799281895</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>25.97599744240152</v>
+        <v>14.98299147498243</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.9192835670113714</v>
+        <v>1.262028859465542</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>16.55457207208008</v>
+        <v>8.898036727459166</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6727</v>
+        <v>6672</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>亞泰金屬</t>
+          <t>騰輝電子-KY</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>498.5467088339622</v>
+        <v>486.1377628952446</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>393</v>
+        <v>264.5</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>51.03994799281895</v>
+        <v>59.94577855775164</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>14.98299147498243</v>
+        <v>21.24094693341862</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.262028859465542</v>
+        <v>1.282461164337962</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>8.898036727459166</v>
+        <v>7.176983530553903</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6672</v>
+        <v>6691</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>騰輝電子-KY</t>
+          <t>洋基工程</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>486.1377628952446</v>
+        <v>480.2728187882935</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>264.5</v>
+        <v>728</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>59.94577855775164</v>
+        <v>55.18303777121351</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>21.24094693341862</v>
+        <v>13.89866219305604</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>1.282461164337962</v>
+        <v>0.6079809346050371</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>7.176983530553903</v>
+        <v>6.998181565526457</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6691</v>
+        <v>6829</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>洋基工程</t>
+          <t>千附精密</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>480.2728187882935</v>
+        <v>479.8690620201465</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>728</v>
+        <v>222</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>55.18303777121351</v>
+        <v>59.50468669503221</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>13.89866219305604</v>
+        <v>16.04722161746431</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.6079809346050371</v>
+        <v>1.348984324244862</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>6.998181565526457</v>
+        <v>4.736439082636447</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6829</v>
+        <v>6510</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>千附精密</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>479.8690620201465</v>
+        <v>477.5415502922536</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>222</v>
+        <v>2820</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>59.50468669503221</v>
+        <v>51.0776328571712</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>16.04722161746431</v>
+        <v>20.70749092967639</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.348984324244862</v>
+        <v>0.9541737437525776</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>4.736439082636447</v>
+        <v>54.09912548711355</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6510</v>
+        <v>6589</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>台康生技</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>477.5415502922536</v>
+        <v>472.2743222588467</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>2820</v>
+        <v>50.8</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.0776328571712</v>
+        <v>60.11889540045873</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>20.70749092967639</v>
+        <v>25.77439845438841</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.9541737437525776</v>
+        <v>0.9450524335911232</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>54.09912548711355</v>
+        <v>0.5729789205672249</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6589</v>
+        <v>6756</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>台康生技</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>472.2743222588467</v>
+        <v>464.7414874519964</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>50.8</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>60.11889540045873</v>
+        <v>54.52769473903533</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>25.77439845438841</v>
+        <v>15.14327173823001</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.9450524335911232</v>
+        <v>0.9164767988572564</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.5729789205672249</v>
+        <v>0.7993497560811187</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6756</v>
+        <v>6504</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>南六</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>464.7414874519964</v>
+        <v>460.414023692824</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>99.90000000000001</v>
+        <v>38.25</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>54.52769473903533</v>
+        <v>50.12902701378209</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>15.14327173823001</v>
+        <v>28.02644348763386</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.9164767988572564</v>
+        <v>0.5291468245191681</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.7993497560811187</v>
+        <v>-0.1533786258226093</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6504</v>
+        <v>6546</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>南六</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>460.414023692824</v>
+        <v>452.4198637867253</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>38.25</v>
+        <v>66</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>50.12902701378209</v>
+        <v>57.78334092921236</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>28.02644348763386</v>
+        <v>30.62753936197033</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.5291468245191681</v>
+        <v>3.787708250970692</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.1533786258226093</v>
+        <v>1.588575306211666</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6546</v>
+        <v>6770</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>452.4198637867253</v>
+        <v>449.7002764429392</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>66</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>57.78334092921236</v>
+        <v>61.26373929911581</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>30.62753936197033</v>
+        <v>15.4769052578571</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>3.787708250970692</v>
+        <v>2.270027644293921</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>1.588575306211666</v>
+        <v>2.13459150476115</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6770</v>
+        <v>6799</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>來頡</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>449.7002764429392</v>
+        <v>440.7172826187211</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>61.26373929911581</v>
+        <v>49.59145046623271</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>15.4769052578571</v>
+        <v>20.05581490893999</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>2.270027644293921</v>
+        <v>0.2829155735352259</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>2.13459150476115</v>
+        <v>1.281423433531484</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6799</v>
+        <v>6505</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>來頡</t>
+          <t>台塑化</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>440.7172826187211</v>
+        <v>438.1793795009783</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>86.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>49.59145046623271</v>
+        <v>50.07855199511643</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>20.05581490893999</v>
+        <v>27.7374494167803</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.2829155735352259</v>
+        <v>0.2177866457636232</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.281423433531484</v>
+        <v>-1.207769330267384</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6505</v>
+        <v>6548</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>台塑化</t>
+          <t>長科*</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>438.1793795009783</v>
+        <v>435.0521483943845</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>69.8</v>
+        <v>74.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>50.07855199511643</v>
+        <v>51.22499969666168</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>27.7374494167803</v>
+        <v>17.11727155639245</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.2177866457636232</v>
+        <v>0.4461786441013731</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.207769330267384</v>
+        <v>1.209274448924492</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6548</v>
+        <v>6530</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>長科*</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>435.0521483943845</v>
+        <v>423.2836128342956</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>74.5</v>
+        <v>85.8</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.22499969666168</v>
+        <v>57.28944619422469</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>17.11727155639245</v>
+        <v>22.59302452956486</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4461786441013731</v>
+        <v>2.834847389957138</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>1.209274448924492</v>
+        <v>2.666565996531028</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6530</v>
+        <v>6526</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>423.2836128342956</v>
+        <v>422.329479933347</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>85.8</v>
+        <v>624</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>57.28944619422469</v>
+        <v>53.83886093575956</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.59302452956486</v>
+        <v>15.35292070175989</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2.834847389957138</v>
+        <v>0.5542136234665451</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>2.666565996531028</v>
+        <v>10.59755789505117</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6526</v>
+        <v>6517</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>保勝光學</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>422.329479933347</v>
+        <v>421.5383526946082</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>624</v>
+        <v>63.7</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.83886093575956</v>
+        <v>47.08100707139351</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>15.35292070175989</v>
+        <v>16.20020864520854</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.5542136234665451</v>
+        <v>0.4652715652574628</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>10.59755789505117</v>
+        <v>-0.0540359291175871</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3071,21 +3071,21 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6517</v>
+        <v>6763</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>保勝光學</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>421.5383526946082</v>
+        <v>410.982191942297</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>63.7</v>
+        <v>42.85</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>47.08100707139351</v>
+        <v>47.82835155718937</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>16.20020864520854</v>
+        <v>25.02419889514221</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.4652715652574628</v>
+        <v>0.4968266866905994</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.0540359291175871</v>
+        <v>0.3283479115650549</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6763</v>
+        <v>6533</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>410.982191942297</v>
+        <v>408.2277726248292</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>42.85</v>
+        <v>249.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>47.82835155718937</v>
+        <v>61.70787743407196</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>25.02419889514221</v>
+        <v>16.565849192008</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4968266866905994</v>
+        <v>0.5453824773727142</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.3283479115650549</v>
+        <v>3.322050141392706</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6533</v>
+        <v>6585</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>鼎基</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>408.2277726248292</v>
+        <v>407.0374625518612</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>249.5</v>
+        <v>120</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>61.70787743407196</v>
+        <v>50.7236559847781</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>16.565849192008</v>
+        <v>16.35072553769538</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.5453824773727142</v>
+        <v>0.4345435613602557</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>3.322050141392706</v>
+        <v>0.360891012927574</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6585</v>
+        <v>6485</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>鼎基</t>
+          <t>點序</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>407.0374625518612</v>
+        <v>392.7865048014315</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>120</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>50.7236559847781</v>
+        <v>49.6143995642172</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>16.35072553769538</v>
+        <v>26.66269260164455</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4345435613602557</v>
+        <v>0.7241540757278374</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.360891012927574</v>
+        <v>1.873941921903262</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6485</v>
+        <v>6592</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>點序</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>392.7865048014315</v>
+        <v>391.4448402195299</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>67.09999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>49.6143995642172</v>
+        <v>55.09629142754447</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>26.66269260164455</v>
+        <v>11.2072472292575</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.7241540757278374</v>
+        <v>0.8069530500899972</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>1.873941921903262</v>
+        <v>0.2185106887053656</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6592</v>
+        <v>6689</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>391.4448402195299</v>
+        <v>389.4192521415363</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>61.7</v>
+        <v>63.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>55.09629142754447</v>
+        <v>54.5499367334045</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.2072472292575</v>
+        <v>21.29307059250384</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.8069530500899972</v>
+        <v>0.8620903063003591</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.2185106887053656</v>
+        <v>0.7531867361078162</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6689</v>
+        <v>6643</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>389.4192521415363</v>
+        <v>387.8861367136258</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>63.5</v>
+        <v>447.5</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>54.5499367334045</v>
+        <v>52.50847002590299</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.29307059250384</v>
+        <v>18.85099116037014</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.8620903063003591</v>
+        <v>0.8842863864963173</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.7531867361078162</v>
+        <v>8.588912875281599</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6643</v>
+        <v>6654</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>天正國際</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>387.8861367136258</v>
+        <v>381.630650104766</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>447.5</v>
+        <v>181</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>52.50847002590299</v>
+        <v>55.53392096478769</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>18.85099116037014</v>
+        <v>18.34462427613047</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.8842863864963173</v>
+        <v>1.155298113260916</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>8.588912875281599</v>
+        <v>1.803078900640267</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6654</v>
+        <v>6640</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>天正國際</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>381.630650104766</v>
+        <v>377.6909510913088</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>181</v>
+        <v>995</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>55.53392096478769</v>
+        <v>53.31723503339638</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>18.34462427613047</v>
+        <v>19.38048023762264</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.155298113260916</v>
+        <v>1.167585064536784</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>1.803078900640267</v>
+        <v>23.69462983223441</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, obv_uptrend, cci_momentum</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6640</v>
+        <v>6666</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>羅麗芬-KY</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>377.6909510913088</v>
+        <v>374.9107921081634</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>995</v>
+        <v>42.65</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>53.31723503339638</v>
+        <v>43.36229981576009</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>19.38048023762264</v>
+        <v>30.87013301758816</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1.167585064536784</v>
+        <v>0.7577976623548421</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>23.69462983223441</v>
+        <v>-0.2598915014942597</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, cci_momentum</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6666</v>
+        <v>6494</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>羅麗芬-KY</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>374.9107921081634</v>
+        <v>372.5334447675029</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>42.65</v>
+        <v>53.9</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>43.36229981576009</v>
+        <v>50.41813117354531</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>30.87013301758816</v>
+        <v>22.41955722586568</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.7577976623548421</v>
+        <v>0.6059778279878705</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.2598915014942597</v>
+        <v>1.121790791764916</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6494</v>
+        <v>6693</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>廣閎科</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>372.5334447675029</v>
+        <v>371.8649085121635</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>53.9</v>
+        <v>185</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,49 +3679,49 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.41813117354531</v>
+        <v>51.00577670198603</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>22.41955722586568</v>
+        <v>22.46103052255724</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.6059778279878705</v>
+        <v>1.497065463783021</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M61" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>1.121790791764916</v>
+        <v>3.192648360741991</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6693</v>
+        <v>6821</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>廣閎科</t>
+          <t>聯寶</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>371.8649085121635</v>
+        <v>371.1482984064796</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>185</v>
+        <v>43</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,49 +3732,49 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>51.00577670198603</v>
+        <v>43.12829268495742</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>22.46103052255724</v>
+        <v>28.16025297565197</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>1.497065463783021</v>
+        <v>1.034965071400752</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M62" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>3.192648360741991</v>
+        <v>0.9324472465659132</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6821</v>
+        <v>6605</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>聯寶</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>371.1482984064796</v>
+        <v>369.3138546373718</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>43</v>
+        <v>136.5</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>43.12829268495742</v>
+        <v>52.75947789678682</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>28.16025297565197</v>
+        <v>12.64831751216909</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.034965071400752</v>
+        <v>0.7222075861351392</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.9324472465659132</v>
+        <v>0.6233162667311183</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6605</v>
+        <v>6706</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>369.3138546373718</v>
+        <v>367.8051387928279</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>136.5</v>
+        <v>122.5</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>52.75947789678682</v>
+        <v>52.3755880663484</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>12.64831751216909</v>
+        <v>23.36460474397057</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.7222075861351392</v>
+        <v>0.8431223528482433</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.6233162667311183</v>
+        <v>4.286729379966468</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6706</v>
+        <v>6577</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>勁豐</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>367.8051387928279</v>
+        <v>362.4222158503363</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>122.5</v>
+        <v>79.5</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>52.3755880663484</v>
+        <v>49.40645441361617</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>23.36460474397057</v>
+        <v>23.08599182028461</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.8431223528482433</v>
+        <v>0.1883145548949289</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>4.286729379966468</v>
+        <v>-0.2670852375813327</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6577</v>
+        <v>6830</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>勁豐</t>
+          <t>汎銓</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>362.4222158503363</v>
+        <v>360.5789029866918</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>79.5</v>
+        <v>420.5</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>49.40645441361617</v>
+        <v>51.47311947012582</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>23.08599182028461</v>
+        <v>19.25641415578155</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.1883145548949289</v>
+        <v>0.980739383128742</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.2670852375813327</v>
+        <v>13.54318826445689</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6830</v>
+        <v>6613</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>汎銓</t>
+          <t>朋億*</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>360.5789029866918</v>
+        <v>356.3800066847713</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>420.5</v>
+        <v>270.5</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.47311947012582</v>
+        <v>41.36222077665525</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>19.25641415578155</v>
+        <v>15.03463185405442</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.980739383128742</v>
+        <v>1.240759642973474</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>13.54318826445689</v>
+        <v>-2.068325791601783</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6613</v>
+        <v>6670</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>朋億*</t>
+          <t>復盛應用</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>356.3800066847713</v>
+        <v>356.3071788874115</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>270.5</v>
+        <v>267</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>41.36222077665525</v>
+        <v>53.39460174768182</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>15.03463185405442</v>
+        <v>12.28256217748137</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1.240759642973474</v>
+        <v>0.665485702499458</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-2.068325791601783</v>
+        <v>0.6848574695101624</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6670</v>
+        <v>6742</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>復盛應用</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>356.3071788874115</v>
+        <v>354.2539102248634</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>267</v>
+        <v>43.9</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>53.39460174768182</v>
+        <v>41.56385898418064</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>12.28256217748137</v>
+        <v>20.56808254848057</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.665485702499458</v>
+        <v>0.3713481851001997</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.6848574695101624</v>
+        <v>0.6645166947290413</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6742</v>
+        <v>6715</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>354.2539102248634</v>
+        <v>353.7694556453644</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>43.9</v>
+        <v>390.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>41.56385898418064</v>
+        <v>51.94378816463318</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>20.56808254848057</v>
+        <v>10.62489755929594</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.3713481851001997</v>
+        <v>1.798540505847586</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.6645166947290413</v>
+        <v>7.231007660877463</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6715</v>
+        <v>6525</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>捷敏-KY</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>353.7694556453644</v>
+        <v>345.720769808407</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>390.5</v>
+        <v>150.5</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>51.94378816463318</v>
+        <v>53.35845739143687</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>10.62489755929594</v>
+        <v>18.72929889450225</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.798540505847586</v>
+        <v>1.412132993746048</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>7.231007660877463</v>
+        <v>1.510925420472423</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6525</v>
+        <v>6531</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>捷敏-KY</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>345.720769808407</v>
+        <v>339.0398904390805</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>150.5</v>
+        <v>865</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,29 +4262,29 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>53.35845739143687</v>
+        <v>50.90411674180633</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>18.72929889450225</v>
+        <v>14.82240748094193</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1.412132993746048</v>
+        <v>0.3109081902483205</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M72" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>1.510925420472423</v>
+        <v>18.76719476341093</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>

</xml_diff>